<commit_message>
regla de faltantes aplicada
</commit_message>
<xml_diff>
--- a/insumos_excel/03- ARQUEOS MF MARZO 2026.xlsx
+++ b/insumos_excel/03- ARQUEOS MF MARZO 2026.xlsx
@@ -22563,9 +22563,6 @@
       <c r="K381" t="n">
         <v>34000000</v>
       </c>
-      <c r="L381" t="n">
-        <v>0</v>
-      </c>
       <c r="M381">
         <f>I381-(H381+J381-K381)- L381</f>
         <v/>
@@ -22623,9 +22620,6 @@
       <c r="K382" t="n">
         <v>800000</v>
       </c>
-      <c r="L382" t="n">
-        <v>10000</v>
-      </c>
       <c r="M382">
         <f>I382-(H382+J382-K382)- L382</f>
         <v/>
@@ -22854,6 +22848,10 @@
       <c r="K386" t="n">
         <v>105999950</v>
       </c>
+      <c r="L386">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M386">
         <f>I386-(H386+J386-K386)- L386</f>
         <v/>
@@ -22906,6 +22904,10 @@
       <c r="K387" t="n">
         <v>199399000</v>
       </c>
+      <c r="L387">
+        <f>-11900000-7385000+133645000</f>
+        <v/>
+      </c>
       <c r="M387">
         <f>I387-(H387+J387-K387)- L387</f>
         <v/>
@@ -22913,6 +22915,11 @@
       <c r="N387">
         <f>IF(M387=0,"Cuadrado",IF(M387&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>Cajero cuadrado, sin observación por parte de la sucursal</t>
+        </is>
       </c>
       <c r="P387" t="n">
         <v>1085303632</v>
@@ -22958,6 +22965,10 @@
       <c r="K388" t="n">
         <v>41872000</v>
       </c>
+      <c r="L388">
+        <f>-490000+610000</f>
+        <v/>
+      </c>
       <c r="M388">
         <f>I388-(H388+J388-K388)- L388</f>
         <v/>
@@ -22965,6 +22976,11 @@
       <c r="N388">
         <f>IF(M388=0,"Cuadrado",IF(M388&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>El faltante $610.000 es cruzado con sobrante contabilizado el día 11/03/2026 ($610.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P388" t="n">
         <v>1129580385</v>
@@ -23010,6 +23026,10 @@
       <c r="K389" t="n">
         <v>53976400</v>
       </c>
+      <c r="L389">
+        <f>150000+220000+155000</f>
+        <v/>
+      </c>
       <c r="M389">
         <f>I389-(H389+J389-K389)- L389</f>
         <v/>
@@ -23017,6 +23037,11 @@
       <c r="N389">
         <f>IF(M389=0,"Cuadrado",IF(M389&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>El faltante $155.000 es cruzado con sobrante contabilizado el día 12/03/2026 ($155.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P389" t="n">
         <v>39447263</v>
@@ -23062,6 +23087,10 @@
       <c r="K390" t="n">
         <v>142716000</v>
       </c>
+      <c r="L390">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M390">
         <f>I390-(H390+J390-K390)- L390</f>
         <v/>
@@ -23114,6 +23143,10 @@
       <c r="K391" t="n">
         <v>0</v>
       </c>
+      <c r="L391">
+        <f>220000</f>
+        <v/>
+      </c>
       <c r="M391">
         <f>I391-(H391+J391-K391)- L391</f>
         <v/>
@@ -23121,6 +23154,11 @@
       <c r="N391">
         <f>IF(M391=0,"Cuadrado",IF(M391&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>El faltante $220.000 es cruzado con sobrante contabilizado el día 11/03/2026 ($220.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P391" t="n">
         <v>79953058</v>
@@ -23166,6 +23204,10 @@
       <c r="K392" t="n">
         <v>2800000</v>
       </c>
+      <c r="L392">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M392">
         <f>I392-(H392+J392-K392)- L392</f>
         <v/>
@@ -23218,6 +23260,10 @@
       <c r="K393" t="n">
         <v>9650000</v>
       </c>
+      <c r="L393">
+        <f>710000</f>
+        <v/>
+      </c>
       <c r="M393">
         <f>I393-(H393+J393-K393)- L393</f>
         <v/>
@@ -23270,6 +23316,10 @@
       <c r="K394" t="n">
         <v>8400000</v>
       </c>
+      <c r="L394">
+        <f>-100000+20000+50000+100000</f>
+        <v/>
+      </c>
       <c r="M394">
         <f>I394-(H394+J394-K394)- L394</f>
         <v/>
@@ -23277,6 +23327,11 @@
       <c r="N394">
         <f>IF(M394=0,"Cuadrado",IF(M394&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>El faltante $170.000 es cruzado con sobrante contabilizado el día 11/03/2026 ($20.000), el día 10/03/2026 ($50.000), el día 06/03/2026 ($100.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P394" t="n">
         <v>79516051</v>
@@ -23322,6 +23377,10 @@
       <c r="K395" t="n">
         <v>53106600</v>
       </c>
+      <c r="L395">
+        <f>2590000+1260000+2970000</f>
+        <v/>
+      </c>
       <c r="M395">
         <f>I395-(H395+J395-K395)- L395</f>
         <v/>
@@ -23374,6 +23433,10 @@
       <c r="K396" t="n">
         <v>15243300</v>
       </c>
+      <c r="L396">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M396">
         <f>I396-(H396+J396-K396)- L396</f>
         <v/>
@@ -23381,6 +23444,11 @@
       <c r="N396">
         <f>IF(M396=0,"Cuadrado",IF(M396&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>Gestión manual - Revisar por el personal encargado</t>
+        </is>
       </c>
       <c r="P396" t="n">
         <v>80386330</v>
@@ -23426,6 +23494,10 @@
       <c r="K397" t="n">
         <v>36080400</v>
       </c>
+      <c r="L397">
+        <f>-1916400</f>
+        <v/>
+      </c>
       <c r="M397">
         <f>I397-(H397+J397-K397)- L397</f>
         <v/>
@@ -23478,6 +23550,10 @@
       <c r="K398" t="n">
         <v>1460000</v>
       </c>
+      <c r="L398">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M398">
         <f>I398-(H398+J398-K398)- L398</f>
         <v/>
@@ -23530,6 +23606,10 @@
       <c r="K399" t="n">
         <v>46141000</v>
       </c>
+      <c r="L399">
+        <f>13715000</f>
+        <v/>
+      </c>
       <c r="M399">
         <f>I399-(H399+J399-K399)- L399</f>
         <v/>
@@ -23582,6 +23662,10 @@
       <c r="K400" t="n">
         <v>0</v>
       </c>
+      <c r="L400">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M400">
         <f>I400-(H400+J400-K400)- L400</f>
         <v/>
@@ -23634,6 +23718,10 @@
       <c r="K401" t="n">
         <v>2100000</v>
       </c>
+      <c r="L401">
+        <f>15150000</f>
+        <v/>
+      </c>
       <c r="M401">
         <f>I401-(H401+J401-K401)- L401</f>
         <v/>
@@ -23641,6 +23729,11 @@
       <c r="N401">
         <f>IF(M401=0,"Cuadrado",IF(M401&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>El faltante $15.150.000 es cruzado con sobrante contabilizado el día 04/03/2026 ($15.150.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P401" t="n">
         <v>1083897578</v>
@@ -23686,6 +23779,10 @@
       <c r="K402" t="n">
         <v>0</v>
       </c>
+      <c r="L402">
+        <f>1995000+1276000+646500</f>
+        <v/>
+      </c>
       <c r="M402">
         <f>I402-(H402+J402-K402)- L402</f>
         <v/>
@@ -23693,6 +23790,11 @@
       <c r="N402">
         <f>IF(M402=0,"Cuadrado",IF(M402&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>El faltante $3.917.500 es cruzado con sobrante contabilizado el día 10/03/2026 ($1.995.000), el día 06/03/2026 ($1.276.000), el día 05/03/2026 ($646.500) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P402" t="n">
         <v>1083897578</v>
@@ -23738,6 +23840,10 @@
       <c r="K403" t="n">
         <v>16583500</v>
       </c>
+      <c r="L403">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M403">
         <f>I403-(H403+J403-K403)- L403</f>
         <v/>
@@ -23790,6 +23896,10 @@
       <c r="K404" t="n">
         <v>18893100</v>
       </c>
+      <c r="L404">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M404">
         <f>I404-(H404+J404-K404)- L404</f>
         <v/>
@@ -23842,6 +23952,10 @@
       <c r="K405" t="n">
         <v>40699600</v>
       </c>
+      <c r="L405">
+        <f>150132000+50000+3600+1400</f>
+        <v/>
+      </c>
       <c r="M405">
         <f>I405-(H405+J405-K405)- L405</f>
         <v/>
@@ -23849,6 +23963,11 @@
       <c r="N405">
         <f>IF(M405=0,"Cuadrado",IF(M405&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>El faltante $55.000 es cruzado con sobrante contabilizado el día 11/03/2026 ($50.000), el día 10/03/2026 ($3.600), el día 06/03/2026 ($1.400) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P405" t="n">
         <v>14697128</v>
@@ -23894,6 +24013,10 @@
       <c r="K406" t="n">
         <v>10484000</v>
       </c>
+      <c r="L406">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M406">
         <f>I406-(H406+J406-K406)- L406</f>
         <v/>
@@ -23946,6 +24069,10 @@
       <c r="K407" t="n">
         <v>28477000</v>
       </c>
+      <c r="L407">
+        <f>12815000</f>
+        <v/>
+      </c>
       <c r="M407">
         <f>I407-(H407+J407-K407)- L407</f>
         <v/>
@@ -23953,6 +24080,11 @@
       <c r="N407">
         <f>IF(M407=0,"Cuadrado",IF(M407&gt;0,"Faltante","Sobrante"))</f>
         <v/>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>El faltante $12.815.000 es cruzado con sobrante contabilizado el día 11/03/2026 ($12.815.000) el cual es reversado por la seccion el día 16/03/2026</t>
+        </is>
       </c>
       <c r="P407" t="n">
         <v>79659379</v>
@@ -23998,6 +24130,10 @@
       <c r="K408" t="n">
         <v>3970000</v>
       </c>
+      <c r="L408">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M408">
         <f>I408-(H408+J408-K408)- L408</f>
         <v/>
@@ -24050,6 +24186,10 @@
       <c r="K409" t="n">
         <v>55430000</v>
       </c>
+      <c r="L409">
+        <f>-880000</f>
+        <v/>
+      </c>
       <c r="M409">
         <f>I409-(H409+J409-K409)- L409</f>
         <v/>
@@ -24102,6 +24242,10 @@
       <c r="K410" t="n">
         <v>9950000</v>
       </c>
+      <c r="L410">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M410">
         <f>I410-(H410+J410-K410)- L410</f>
         <v/>
@@ -24154,6 +24298,10 @@
       <c r="K411" t="n">
         <v>0</v>
       </c>
+      <c r="L411">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M411">
         <f>I411-(H411+J411-K411)- L411</f>
         <v/>
@@ -24206,6 +24354,10 @@
       <c r="K412" t="n">
         <v>33723000</v>
       </c>
+      <c r="L412">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M412">
         <f>I412-(H412+J412-K412)- L412</f>
         <v/>
@@ -24258,6 +24410,10 @@
       <c r="K413" t="n">
         <v>16331000</v>
       </c>
+      <c r="L413">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M413">
         <f>I413-(H413+J413-K413)- L413</f>
         <v/>
@@ -24310,6 +24466,10 @@
       <c r="K414" t="n">
         <v>53010000</v>
       </c>
+      <c r="L414">
+        <f>0</f>
+        <v/>
+      </c>
       <c r="M414">
         <f>I414-(H414+J414-K414)- L414</f>
         <v/>
@@ -24362,6 +24522,10 @@
       <c r="K415" t="n">
         <v>20370000</v>
       </c>
+      <c r="L415">
+        <f>1377400</f>
+        <v/>
+      </c>
       <c r="M415">
         <f>I415-(H415+J415-K415)- L415</f>
         <v/>
@@ -24414,8 +24578,9 @@
       <c r="K416" t="n">
         <v>7895000</v>
       </c>
-      <c r="L416" t="n">
-        <v>0</v>
+      <c r="L416">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M416">
         <f>I416-(H416+J416-K416)- L416</f>
@@ -24474,8 +24639,9 @@
       <c r="K417" t="n">
         <v>28766000</v>
       </c>
-      <c r="L417" t="n">
-        <v>0</v>
+      <c r="L417">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M417">
         <f>I417-(H417+J417-K417)- L417</f>
@@ -24534,8 +24700,9 @@
       <c r="K418" t="n">
         <v>6200000</v>
       </c>
-      <c r="L418" t="n">
-        <v>0</v>
+      <c r="L418">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M418">
         <f>I418-(H418+J418-K418)- L418</f>
@@ -24594,8 +24761,9 @@
       <c r="K419" t="n">
         <v>0</v>
       </c>
-      <c r="L419" t="n">
-        <v>0</v>
+      <c r="L419">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M419">
         <f>I419-(H419+J419-K419)- L419</f>
@@ -24654,8 +24822,9 @@
       <c r="K420" t="n">
         <v>0</v>
       </c>
-      <c r="L420" t="n">
-        <v>0</v>
+      <c r="L420">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M420">
         <f>I420-(H420+J420-K420)- L420</f>
@@ -24714,8 +24883,9 @@
       <c r="K421" t="n">
         <v>159780000</v>
       </c>
-      <c r="L421" t="n">
-        <v>0</v>
+      <c r="L421">
+        <f>0</f>
+        <v/>
       </c>
       <c r="M421">
         <f>I421-(H421+J421-K421)- L421</f>
@@ -35165,7 +35335,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
@@ -35271,8 +35440,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -35291,7 +35458,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -35334,7 +35500,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -35342,8 +35507,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -35351,586 +35514,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
     <row r="611">
       <c r="G611" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
De sobrantes se toma primero DIARIOS. No repetir arc consecutivo
</commit_message>
<xml_diff>
--- a/insumos_excel/03- ARQUEOS MF MARZO 2026.xlsx
+++ b/insumos_excel/03- ARQUEOS MF MARZO 2026.xlsx
@@ -30478,7 +30478,7 @@
       </c>
       <c r="O519" t="inlineStr">
         <is>
-          <t>ACLARAR DIFERENCIA Y REPETIR EL ARQUEO</t>
+          <t>La diferencia es contabilizada por la Gerencia De Autoservicios y Efectivo de manera centralizada a la cuenta de faltantes 168710093 el 18/03/2026, esta diferencia ingresa a proceso de investigación en el área para identificar a que corresponde.</t>
         </is>
       </c>
     </row>
@@ -30871,7 +30871,7 @@
         <v>13595100</v>
       </c>
       <c r="L526">
-        <f>3320000+53950</f>
+        <f>399900+1800000+1174050</f>
         <v/>
       </c>
       <c r="M526">
@@ -30884,7 +30884,7 @@
       </c>
       <c r="O526" t="inlineStr">
         <is>
-          <t>El faltante $3.373.950 es cruzado con sobrante contabilizado el día 10/03/2026 ($3.320.000), el día 11/03/2026 ($53.950) el cual es reversado por la seccion el día 18/03/2026</t>
+          <t>El faltante $3.373.950 es cruzado con sobrante contabilizado el día 11/03/2026 ($399.900), el día 12/03/2026 ($1.800.000), el día 13/03/2026 ($1.174.050) el cual es reversado por la seccion el día 18/03/2026</t>
         </is>
       </c>
     </row>
@@ -31219,7 +31219,7 @@
         <v>36755000</v>
       </c>
       <c r="L532">
-        <f>0</f>
+        <f>490000</f>
         <v/>
       </c>
       <c r="M532">
@@ -31232,7 +31232,7 @@
       </c>
       <c r="O532" t="inlineStr">
         <is>
-          <t>ACLARAR DIFERENCIA Y REPETIR EL ARQUEO</t>
+          <t>El faltante $490.000 es cruzado con sobrante contabilizado el día 04/03/2026 ($490.000) el cual es reversado por la seccion el día 18/03/2026</t>
         </is>
       </c>
     </row>
@@ -31915,7 +31915,7 @@
         <v>63093050</v>
       </c>
       <c r="L544">
-        <f>-260050</f>
+        <f>-260050+310000+880000+190000+10000</f>
         <v/>
       </c>
       <c r="M544">
@@ -31928,7 +31928,7 @@
       </c>
       <c r="O544" t="inlineStr">
         <is>
-          <t>ACLARAR DIFERENCIA Y REPETIR EL ARQUEO</t>
+          <t>El faltante $1.390.000 es cruzado con sobrante contabilizado el día 04/03/2026 ($310.000), el día 06/03/2026 ($880.000), el día 10/03/2026 ($190.000), el día 11/03/2026 ($10.000) el cual es reversado por la seccion el día 18/03/2026</t>
         </is>
       </c>
     </row>

</xml_diff>